<commit_message>
SOP and laser safety
</commit_message>
<xml_diff>
--- a/Equipment/Inventory.xlsx
+++ b/Equipment/Inventory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\physics-svc-yuta\Documents\Takahashi Lab\Equipment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE69ABE0-9B74-43DE-9799-0C13E806987E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B21C7E-637D-4A74-8213-6C666D2AEE86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="Software" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -247,9 +248,6 @@
     <t>LA-01 IR FC</t>
   </si>
   <si>
-    <t>1064 nm Laser</t>
-  </si>
-  <si>
     <t>F-01 A</t>
   </si>
   <si>
@@ -274,9 +272,6 @@
     <t>Scanning TCT data acquisition</t>
   </si>
   <si>
-    <t>50 mW, fiber coupled</t>
-  </si>
-  <si>
     <t>Standa</t>
   </si>
   <si>
@@ -308,6 +303,12 @@
   </si>
   <si>
     <t>consists of 8SMC5-USB-B8-1 and 8SMC5-USB-B9-2</t>
+  </si>
+  <si>
+    <t>Laser</t>
+  </si>
+  <si>
+    <t>1064 nm, 50 mW, fiber coupled</t>
   </si>
 </sst>
 </file>
@@ -1092,10 +1093,10 @@
         <v>72</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="F20" s="5">
         <v>1</v>
@@ -1109,13 +1110,13 @@
         <v>62</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="F21" s="5">
         <v>1</v>
@@ -1126,16 +1127,16 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="D22" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F22" s="5">
         <v>1</v>
@@ -1143,16 +1144,16 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="D23" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="F23" s="5">
         <v>1</v>
@@ -1160,16 +1161,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="F24" s="5">
         <v>1</v>
@@ -1252,13 +1253,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>79</v>
-      </c>
       <c r="C1" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>8</v>
@@ -1278,7 +1279,7 @@
         <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>19</v>
@@ -1289,7 +1290,7 @@
         <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
updates TCT software and cad box
</commit_message>
<xml_diff>
--- a/Equipment/Inventory.xlsx
+++ b/Equipment/Inventory.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\physics-svc-yuta\Documents\Takahashi Lab\Equipment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B21C7E-637D-4A74-8213-6C666D2AEE86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818401CB-4603-4CCA-82E9-8D1D0CB3FEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hardware" sheetId="1" r:id="rId1"/>
     <sheet name="Software" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="102">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -266,9 +265,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Particlars laser control</t>
-  </si>
-  <si>
     <t>Scanning TCT data acquisition</t>
   </si>
   <si>
@@ -309,6 +305,33 @@
   </si>
   <si>
     <t>1064 nm, 50 mW, fiber coupled</t>
+  </si>
+  <si>
+    <t>Xilinx</t>
+  </si>
+  <si>
+    <t>Kintex HW-KC705</t>
+  </si>
+  <si>
+    <t>1165</t>
+  </si>
+  <si>
+    <t>Whizzsystems SN: 604031951839-92389</t>
+  </si>
+  <si>
+    <t>FPGA</t>
+  </si>
+  <si>
+    <t>TCTAnalyse</t>
+  </si>
+  <si>
+    <t>ParticlarsLaserControl</t>
+  </si>
+  <si>
+    <t>PSTCT</t>
+  </si>
+  <si>
+    <t>ROOT library for analysis of TCT data</t>
   </si>
 </sst>
 </file>
@@ -361,7 +384,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -376,6 +399,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -657,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31" style="1" customWidth="1"/>
@@ -1028,7 +1054,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>62</v>
       </c>
@@ -1045,7 +1071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>62</v>
       </c>
@@ -1065,7 +1091,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>62</v>
       </c>
@@ -1085,7 +1111,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>62</v>
       </c>
@@ -1093,10 +1119,10 @@
         <v>72</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="F20" s="5">
         <v>1</v>
@@ -1105,7 +1131,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>62</v>
       </c>
@@ -1125,58 +1151,78 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="C22" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="D22" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F22" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>87</v>
       </c>
       <c r="F23" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="F24" s="5">
         <v>1</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F25" s="5">
+        <v>1</v>
+      </c>
+      <c r="I25" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1228,9 +1274,10 @@
     <hyperlink ref="B23" r:id="rId45" xr:uid="{08092570-B280-4648-AC91-34AB2EF99F76}"/>
     <hyperlink ref="G24" r:id="rId46" xr:uid="{C2F26245-31D0-43EC-AFA5-75568258EC14}"/>
     <hyperlink ref="B24" r:id="rId47" xr:uid="{F709732C-BD0E-4DC2-B814-DBA5C76BA3B9}"/>
+    <hyperlink ref="B25" r:id="rId48" xr:uid="{CF9B53CF-B0C2-4222-B48F-4B35DF285DC5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId48"/>
+  <pageSetup orientation="portrait" r:id="rId49"/>
   <ignoredErrors>
     <ignoredError sqref="B11" numberStoredAsText="1"/>
   </ignoredErrors>
@@ -1239,14 +1286,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B6C3D6-DB6D-431B-A312-06E15229C9CC}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" customWidth="1"/>
     <col min="2" max="2" width="30.5703125" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
     <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
+    <col min="5" max="5" width="28.42578125" customWidth="1"/>
     <col min="6" max="6" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1279,7 +1326,10 @@
         <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>99</v>
+      </c>
+      <c r="C2">
+        <v>2.1</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>19</v>
@@ -1290,9 +1340,32 @@
         <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <v>3.2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>79</v>
       </c>
       <c r="F3" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1300,6 +1373,7 @@
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{D659E979-CDB6-4651-80D9-1A245A451744}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{D45BCB81-7288-49BE-8B44-DF27A6334EC7}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{6EF7B9FF-3C26-4147-871B-25791246E6CE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>